<commit_message>
Harden spreadsheet peek support claims
</commit_message>
<xml_diff>
--- a/examples/sample-financials.xlsx
+++ b/examples/sample-financials.xlsx
@@ -18,7 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -48,8 +50,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -933,15 +936,11 @@
           <t>Account</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Mar 31 2024</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Dec 31 2023</t>
-        </is>
+      <c r="B1" s="1" t="n">
+        <v>45382</v>
+      </c>
+      <c r="C1" s="1" t="n">
+        <v>45291</v>
       </c>
       <c r="D1" t="inlineStr">
         <is>

</xml_diff>